<commit_message>
API in Mihai folder
</commit_message>
<xml_diff>
--- a/Mihai/CLI-backend/databases/PostDatabase.xlsx
+++ b/Mihai/CLI-backend/databases/PostDatabase.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\serba\AppData\Roaming\SPB_Data\ZTH-Team-Deltaspace\App\CLI-backend\databases\"/>
     </mc:Choice>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>ID</t>
   </si>
@@ -41,12 +41,34 @@
   </si>
   <si>
     <t>NSFW</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Mihai14</t>
+  </si>
+  <si>
+    <t>MyPostTitle</t>
+  </si>
+  <si>
+    <t>MyPostContnets</t>
+  </si>
+  <si>
+    <t>No image link</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>true</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -412,39 +434,62 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="2.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="7.2109375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="10.3046875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="14.10546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="11.80859375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="10.0078125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="6.20703125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>6</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>